<commit_message>
remove bold from tables
</commit_message>
<xml_diff>
--- a/results/02_4tier_filtering/02_top9_cohort_comprehensive_analysis.xlsx
+++ b/results/02_4tier_filtering/02_top9_cohort_comprehensive_analysis.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Top9_Master_Census" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Top9_Macro_Summary_vs_Top25" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Top9_Cluster_Archetypes" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Top9_Econometric_Relationships" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="TSA_Annual_Throughput" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="TSA_Recovery_Pct_2019_Base" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Sched_Departures_Annual" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Sched_Recovery_Pct_2019_Base" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Temporal_Regime_Coupling" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Hourly_Lead_Lag_Transfer" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top9_Master_Census" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top9_Macro_Summary_vs_Top25" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top9_Cluster_Archetypes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top9_Econometric_Relationships" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TSA_Annual_Throughput" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TSA_Recovery_Pct_2019_Base" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sched_Departures_Annual" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sched_Recovery_Pct_2019_Base" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Temporal_Regime_Coupling" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hourly_Lead_Lag_Transfer" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>